<commit_message>
Change from sero to iris colour
</commit_message>
<xml_diff>
--- a/data/RawData/metadata_2005-2023.xlsx
+++ b/data/RawData/metadata_2005-2023.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ponchon\Documents\Projects\NorthernGannets2023\Analysis\NorthernGannets2023\data\RawData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aponchon\Nextcloud\Aurore\Projects\NorthernGannets2023\Analysis\NorthernGannets2023\data\RawData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D16D3D7-9725-4547-9C52-E27657C3934B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6630DF76-DA50-409A-8C80-30113FDDEFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{180F53A7-9CD1-4793-8959-A57DB5048E36}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{180F53A7-9CD1-4793-8959-A57DB5048E36}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="372">
   <si>
     <t>year</t>
   </si>
@@ -1130,6 +1130,30 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Yeux_bino</t>
+  </si>
+  <si>
+    <t>Yeux_colo</t>
+  </si>
+  <si>
+    <t>1dark</t>
+  </si>
+  <si>
+    <t>2dark</t>
+  </si>
+  <si>
+    <t>2spotted</t>
+  </si>
+  <si>
+    <t>2white</t>
+  </si>
+  <si>
+    <t>1spotted</t>
+  </si>
+  <si>
+    <t>1dark1spotted</t>
   </si>
 </sst>
 </file>
@@ -1139,7 +1163,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1177,13 +1201,6 @@
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1300,7 +1317,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1416,7 +1433,6 @@
     <xf numFmtId="164" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1754,7 +1770,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACFEFB18-4BDE-42FE-B8C4-54C00AF18A71}">
-  <dimension ref="A1:O241"/>
+  <dimension ref="A1:Q241"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="11.42578125" style="2"/>
@@ -1762,7 +1778,7 @@
     <col min="5" max="12" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
@@ -1803,13 +1819,19 @@
         <v>354</v>
       </c>
       <c r="N1" s="25" t="s">
+        <v>364</v>
+      </c>
+      <c r="O1" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="P1" s="25" t="s">
         <v>355</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="Q1" s="25" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2022</v>
       </c>
@@ -1839,8 +1861,10 @@
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2022</v>
       </c>
@@ -1872,8 +1896,10 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2022</v>
       </c>
@@ -1905,8 +1931,10 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2022</v>
       </c>
@@ -1938,8 +1966,10 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2022</v>
       </c>
@@ -1971,8 +2001,10 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2022</v>
       </c>
@@ -2004,8 +2036,10 @@
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>2022</v>
       </c>
@@ -2037,8 +2071,10 @@
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>2022</v>
       </c>
@@ -2070,8 +2106,10 @@
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>2022</v>
       </c>
@@ -2103,8 +2141,10 @@
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>2022</v>
       </c>
@@ -2136,8 +2176,10 @@
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>2022</v>
       </c>
@@ -2169,8 +2211,10 @@
       <c r="M12" s="3"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>2022</v>
       </c>
@@ -2202,8 +2246,10 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>2022</v>
       </c>
@@ -2235,8 +2281,10 @@
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>2022</v>
       </c>
@@ -2268,8 +2316,10 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>2022</v>
       </c>
@@ -2301,8 +2351,10 @@
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>2005</v>
       </c>
@@ -2326,8 +2378,10 @@
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
       <c r="O17" s="6"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>2005</v>
       </c>
@@ -2353,8 +2407,10 @@
       <c r="M18" s="6"/>
       <c r="N18" s="6"/>
       <c r="O18" s="6"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>2005</v>
       </c>
@@ -2380,8 +2436,10 @@
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>2005</v>
       </c>
@@ -2407,8 +2465,10 @@
       <c r="M20" s="6"/>
       <c r="N20" s="6"/>
       <c r="O20" s="6"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>2005</v>
       </c>
@@ -2432,8 +2492,10 @@
       <c r="M21" s="6"/>
       <c r="N21" s="6"/>
       <c r="O21" s="6"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>2005</v>
       </c>
@@ -2457,8 +2519,10 @@
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
       <c r="O22" s="6"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>2005</v>
       </c>
@@ -2482,8 +2546,10 @@
       <c r="M23" s="6"/>
       <c r="N23" s="6"/>
       <c r="O23" s="6"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>2005</v>
       </c>
@@ -2507,8 +2573,10 @@
       <c r="M24" s="6"/>
       <c r="N24" s="6"/>
       <c r="O24" s="6"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>2005</v>
       </c>
@@ -2532,8 +2600,10 @@
       <c r="M25" s="6"/>
       <c r="N25" s="6"/>
       <c r="O25" s="6"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <v>2005</v>
       </c>
@@ -2557,8 +2627,10 @@
       <c r="M26" s="6"/>
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>2005</v>
       </c>
@@ -2584,8 +2656,10 @@
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>2005</v>
       </c>
@@ -2609,8 +2683,10 @@
       <c r="M28" s="6"/>
       <c r="N28" s="6"/>
       <c r="O28" s="6"/>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>2005</v>
       </c>
@@ -2636,8 +2712,10 @@
       <c r="M29" s="6"/>
       <c r="N29" s="6"/>
       <c r="O29" s="6"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>2005</v>
       </c>
@@ -2661,8 +2739,10 @@
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>2005</v>
       </c>
@@ -2686,8 +2766,10 @@
       <c r="M31" s="6"/>
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>2005</v>
       </c>
@@ -2711,8 +2793,10 @@
       <c r="M32" s="6"/>
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>2005</v>
       </c>
@@ -2736,8 +2820,10 @@
       <c r="M33" s="6"/>
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>2005</v>
       </c>
@@ -2761,8 +2847,10 @@
       <c r="M34" s="6"/>
       <c r="N34" s="6"/>
       <c r="O34" s="6"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>2005</v>
       </c>
@@ -2788,8 +2876,10 @@
       <c r="M35" s="6"/>
       <c r="N35" s="6"/>
       <c r="O35" s="6"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P35" s="6"/>
+      <c r="Q35" s="6"/>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>2005</v>
       </c>
@@ -2813,8 +2903,10 @@
       <c r="M36" s="6"/>
       <c r="N36" s="6"/>
       <c r="O36" s="6"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6"/>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>2005</v>
       </c>
@@ -2840,8 +2932,10 @@
       <c r="M37" s="6"/>
       <c r="N37" s="6"/>
       <c r="O37" s="6"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6"/>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="8">
         <v>2006</v>
       </c>
@@ -2867,8 +2961,10 @@
       <c r="M38" s="8"/>
       <c r="N38" s="8"/>
       <c r="O38" s="8"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="8">
         <v>2006</v>
       </c>
@@ -2895,8 +2991,10 @@
       <c r="M39" s="8"/>
       <c r="N39" s="8"/>
       <c r="O39" s="8"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>2006</v>
       </c>
@@ -2923,8 +3021,10 @@
       <c r="M40" s="8"/>
       <c r="N40" s="8"/>
       <c r="O40" s="8"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P40" s="8"/>
+      <c r="Q40" s="8"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="8">
         <v>2006</v>
       </c>
@@ -2950,8 +3050,10 @@
       <c r="M41" s="8"/>
       <c r="N41" s="8"/>
       <c r="O41" s="8"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P41" s="8"/>
+      <c r="Q41" s="8"/>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>2006</v>
       </c>
@@ -2977,8 +3079,10 @@
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
       <c r="O42" s="8"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P42" s="8"/>
+      <c r="Q42" s="8"/>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="8">
         <v>2006</v>
       </c>
@@ -3005,8 +3109,10 @@
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
       <c r="O43" s="8"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P43" s="8"/>
+      <c r="Q43" s="8"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="8">
         <v>2006</v>
       </c>
@@ -3032,8 +3138,10 @@
       <c r="M44" s="8"/>
       <c r="N44" s="8"/>
       <c r="O44" s="8"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P44" s="8"/>
+      <c r="Q44" s="8"/>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="8">
         <v>2006</v>
       </c>
@@ -3060,8 +3168,10 @@
       <c r="M45" s="8"/>
       <c r="N45" s="8"/>
       <c r="O45" s="8"/>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P45" s="8"/>
+      <c r="Q45" s="8"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>2006</v>
       </c>
@@ -3087,8 +3197,10 @@
       <c r="M46" s="8"/>
       <c r="N46" s="8"/>
       <c r="O46" s="8"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P46" s="8"/>
+      <c r="Q46" s="8"/>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>2006</v>
       </c>
@@ -3115,8 +3227,10 @@
       <c r="M47" s="8"/>
       <c r="N47" s="8"/>
       <c r="O47" s="8"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P47" s="8"/>
+      <c r="Q47" s="8"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="8">
         <v>2006</v>
       </c>
@@ -3143,8 +3257,10 @@
       <c r="M48" s="8"/>
       <c r="N48" s="8"/>
       <c r="O48" s="8"/>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P48" s="8"/>
+      <c r="Q48" s="8"/>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="8">
         <v>2006</v>
       </c>
@@ -3171,8 +3287,10 @@
       <c r="M49" s="8"/>
       <c r="N49" s="8"/>
       <c r="O49" s="8"/>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P49" s="8"/>
+      <c r="Q49" s="8"/>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>2006</v>
       </c>
@@ -3198,8 +3316,10 @@
       <c r="M50" s="8"/>
       <c r="N50" s="8"/>
       <c r="O50" s="8"/>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P50" s="8"/>
+      <c r="Q50" s="8"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>2006</v>
       </c>
@@ -3226,8 +3346,10 @@
       <c r="M51" s="8"/>
       <c r="N51" s="8"/>
       <c r="O51" s="8"/>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P51" s="8"/>
+      <c r="Q51" s="8"/>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <v>2006</v>
       </c>
@@ -3253,8 +3375,10 @@
       <c r="M52" s="8"/>
       <c r="N52" s="8"/>
       <c r="O52" s="8"/>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P52" s="8"/>
+      <c r="Q52" s="8"/>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="8">
         <v>2006</v>
       </c>
@@ -3281,8 +3405,10 @@
       <c r="M53" s="8"/>
       <c r="N53" s="8"/>
       <c r="O53" s="8"/>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P53" s="8"/>
+      <c r="Q53" s="8"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="8">
         <v>2006</v>
       </c>
@@ -3309,8 +3435,10 @@
       <c r="M54" s="8"/>
       <c r="N54" s="8"/>
       <c r="O54" s="8"/>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P54" s="8"/>
+      <c r="Q54" s="8"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="8">
         <v>2006</v>
       </c>
@@ -3336,8 +3464,10 @@
       <c r="M55" s="8"/>
       <c r="N55" s="8"/>
       <c r="O55" s="8"/>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P55" s="8"/>
+      <c r="Q55" s="8"/>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>2006</v>
       </c>
@@ -3364,8 +3494,10 @@
       <c r="M56" s="8"/>
       <c r="N56" s="8"/>
       <c r="O56" s="8"/>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P56" s="8"/>
+      <c r="Q56" s="8"/>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>2006</v>
       </c>
@@ -3392,8 +3524,10 @@
       <c r="M57" s="8"/>
       <c r="N57" s="8"/>
       <c r="O57" s="8"/>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P57" s="8"/>
+      <c r="Q57" s="8"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="9">
         <v>2010</v>
       </c>
@@ -3425,8 +3559,10 @@
       <c r="M58" s="19"/>
       <c r="N58" s="19"/>
       <c r="O58" s="19"/>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P58" s="19"/>
+      <c r="Q58" s="19"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="9">
         <v>2010</v>
       </c>
@@ -3458,8 +3594,10 @@
       <c r="M59" s="19"/>
       <c r="N59" s="19"/>
       <c r="O59" s="19"/>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P59" s="19"/>
+      <c r="Q59" s="19"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="9">
         <v>2010</v>
       </c>
@@ -3493,8 +3631,10 @@
       <c r="M60" s="19"/>
       <c r="N60" s="19"/>
       <c r="O60" s="19"/>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P60" s="19"/>
+      <c r="Q60" s="19"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="9">
         <v>2010</v>
       </c>
@@ -3528,8 +3668,10 @@
       <c r="M61" s="19"/>
       <c r="N61" s="19"/>
       <c r="O61" s="19"/>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P61" s="19"/>
+      <c r="Q61" s="19"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="9">
         <v>2010</v>
       </c>
@@ -3563,8 +3705,10 @@
       <c r="M62" s="19"/>
       <c r="N62" s="19"/>
       <c r="O62" s="19"/>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P62" s="19"/>
+      <c r="Q62" s="19"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="9">
         <v>2010</v>
       </c>
@@ -3598,8 +3742,10 @@
       <c r="M63" s="19"/>
       <c r="N63" s="19"/>
       <c r="O63" s="19"/>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P63" s="19"/>
+      <c r="Q63" s="19"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="9">
         <v>2010</v>
       </c>
@@ -3633,8 +3779,10 @@
       <c r="M64" s="19"/>
       <c r="N64" s="19"/>
       <c r="O64" s="19"/>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P64" s="19"/>
+      <c r="Q64" s="19"/>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="9">
         <v>2010</v>
       </c>
@@ -3666,8 +3814,10 @@
       <c r="M65" s="19"/>
       <c r="N65" s="19"/>
       <c r="O65" s="19"/>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P65" s="19"/>
+      <c r="Q65" s="19"/>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="9">
         <v>2010</v>
       </c>
@@ -3701,8 +3851,10 @@
       <c r="M66" s="19"/>
       <c r="N66" s="19"/>
       <c r="O66" s="19"/>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P66" s="19"/>
+      <c r="Q66" s="19"/>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="9">
         <v>2010</v>
       </c>
@@ -3736,8 +3888,10 @@
       <c r="M67" s="19"/>
       <c r="N67" s="19"/>
       <c r="O67" s="19"/>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P67" s="19"/>
+      <c r="Q67" s="19"/>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="9">
         <v>2010</v>
       </c>
@@ -3769,8 +3923,10 @@
       <c r="M68" s="19"/>
       <c r="N68" s="19"/>
       <c r="O68" s="19"/>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P68" s="19"/>
+      <c r="Q68" s="19"/>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="9">
         <v>2010</v>
       </c>
@@ -3802,8 +3958,10 @@
       <c r="M69" s="19"/>
       <c r="N69" s="19"/>
       <c r="O69" s="19"/>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P69" s="19"/>
+      <c r="Q69" s="19"/>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>2010</v>
       </c>
@@ -3837,8 +3995,10 @@
       <c r="M70" s="19"/>
       <c r="N70" s="19"/>
       <c r="O70" s="19"/>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P70" s="19"/>
+      <c r="Q70" s="19"/>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="9">
         <v>2010</v>
       </c>
@@ -3870,8 +4030,10 @@
       <c r="M71" s="19"/>
       <c r="N71" s="19"/>
       <c r="O71" s="19"/>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P71" s="19"/>
+      <c r="Q71" s="19"/>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="9">
         <v>2010</v>
       </c>
@@ -3905,8 +4067,10 @@
       <c r="M72" s="19"/>
       <c r="N72" s="19"/>
       <c r="O72" s="19"/>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P72" s="19"/>
+      <c r="Q72" s="19"/>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="9">
         <v>2010</v>
       </c>
@@ -3936,8 +4100,10 @@
       <c r="M73" s="19"/>
       <c r="N73" s="19"/>
       <c r="O73" s="19"/>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P73" s="19"/>
+      <c r="Q73" s="19"/>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="9">
         <v>2010</v>
       </c>
@@ -3965,8 +4131,10 @@
       <c r="M74" s="19"/>
       <c r="N74" s="19"/>
       <c r="O74" s="19"/>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P74" s="19"/>
+      <c r="Q74" s="19"/>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="9">
         <v>2010</v>
       </c>
@@ -3996,8 +4164,10 @@
       <c r="M75" s="19"/>
       <c r="N75" s="19"/>
       <c r="O75" s="19"/>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P75" s="19"/>
+      <c r="Q75" s="19"/>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="9">
         <v>2010</v>
       </c>
@@ -4031,8 +4201,10 @@
       <c r="M76" s="19"/>
       <c r="N76" s="19"/>
       <c r="O76" s="19"/>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P76" s="19"/>
+      <c r="Q76" s="19"/>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="9">
         <v>2010</v>
       </c>
@@ -4064,8 +4236,10 @@
       <c r="M77" s="19"/>
       <c r="N77" s="19"/>
       <c r="O77" s="19"/>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P77" s="19"/>
+      <c r="Q77" s="19"/>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="9">
         <v>2010</v>
       </c>
@@ -4099,8 +4273,10 @@
       <c r="M78" s="19"/>
       <c r="N78" s="19"/>
       <c r="O78" s="19"/>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P78" s="19"/>
+      <c r="Q78" s="19"/>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="9">
         <v>2010</v>
       </c>
@@ -4130,8 +4306,10 @@
       <c r="M79" s="19"/>
       <c r="N79" s="19"/>
       <c r="O79" s="19"/>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P79" s="19"/>
+      <c r="Q79" s="19"/>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="11">
         <v>2011</v>
       </c>
@@ -4167,8 +4345,10 @@
       <c r="M80" s="11"/>
       <c r="N80" s="11"/>
       <c r="O80" s="11"/>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P80" s="11"/>
+      <c r="Q80" s="11"/>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="11">
         <v>2011</v>
       </c>
@@ -4204,8 +4384,10 @@
       <c r="M81" s="11"/>
       <c r="N81" s="11"/>
       <c r="O81" s="11"/>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P81" s="11"/>
+      <c r="Q81" s="11"/>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="11">
         <v>2011</v>
       </c>
@@ -4241,8 +4423,10 @@
       <c r="M82" s="11"/>
       <c r="N82" s="11"/>
       <c r="O82" s="11"/>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P82" s="11"/>
+      <c r="Q82" s="11"/>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="11">
         <v>2011</v>
       </c>
@@ -4278,8 +4462,10 @@
       <c r="M83" s="11"/>
       <c r="N83" s="11"/>
       <c r="O83" s="11"/>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P83" s="11"/>
+      <c r="Q83" s="11"/>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="11">
         <v>2011</v>
       </c>
@@ -4315,8 +4501,10 @@
       <c r="M84" s="11"/>
       <c r="N84" s="11"/>
       <c r="O84" s="11"/>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P84" s="11"/>
+      <c r="Q84" s="11"/>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="11">
         <v>2011</v>
       </c>
@@ -4354,8 +4542,10 @@
       <c r="M85" s="11"/>
       <c r="N85" s="11"/>
       <c r="O85" s="11"/>
-    </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P85" s="11"/>
+      <c r="Q85" s="11"/>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="11">
         <v>2011</v>
       </c>
@@ -4391,8 +4581,10 @@
       <c r="M86" s="11"/>
       <c r="N86" s="11"/>
       <c r="O86" s="11"/>
-    </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P86" s="11"/>
+      <c r="Q86" s="11"/>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="11">
         <v>2011</v>
       </c>
@@ -4429,8 +4621,10 @@
       <c r="M87" s="11"/>
       <c r="N87" s="11"/>
       <c r="O87" s="11"/>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P87" s="11"/>
+      <c r="Q87" s="11"/>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="11">
         <v>2011</v>
       </c>
@@ -4466,8 +4660,10 @@
       <c r="M88" s="11"/>
       <c r="N88" s="11"/>
       <c r="O88" s="11"/>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P88" s="11"/>
+      <c r="Q88" s="11"/>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="11">
         <v>2011</v>
       </c>
@@ -4503,8 +4699,10 @@
       <c r="M89" s="11"/>
       <c r="N89" s="11"/>
       <c r="O89" s="11"/>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P89" s="11"/>
+      <c r="Q89" s="11"/>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="11">
         <v>2011</v>
       </c>
@@ -4542,8 +4740,10 @@
       <c r="M90" s="11"/>
       <c r="N90" s="11"/>
       <c r="O90" s="11"/>
-    </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P90" s="11"/>
+      <c r="Q90" s="11"/>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="11">
         <v>2011</v>
       </c>
@@ -4579,8 +4779,10 @@
       <c r="M91" s="11"/>
       <c r="N91" s="11"/>
       <c r="O91" s="11"/>
-    </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P91" s="11"/>
+      <c r="Q91" s="11"/>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="11">
         <v>2011</v>
       </c>
@@ -4616,8 +4818,10 @@
       <c r="M92" s="11"/>
       <c r="N92" s="11"/>
       <c r="O92" s="11"/>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P92" s="11"/>
+      <c r="Q92" s="11"/>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="11">
         <v>2011</v>
       </c>
@@ -4645,8 +4849,10 @@
       <c r="M93" s="11"/>
       <c r="N93" s="11"/>
       <c r="O93" s="11"/>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P93" s="11"/>
+      <c r="Q93" s="11"/>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="11">
         <v>2011</v>
       </c>
@@ -4682,8 +4888,10 @@
       <c r="M94" s="11"/>
       <c r="N94" s="11"/>
       <c r="O94" s="11"/>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P94" s="11"/>
+      <c r="Q94" s="11"/>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="11">
         <v>2011</v>
       </c>
@@ -4719,8 +4927,10 @@
       <c r="M95" s="11"/>
       <c r="N95" s="11"/>
       <c r="O95" s="11"/>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P95" s="11"/>
+      <c r="Q95" s="11"/>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="11">
         <v>2011</v>
       </c>
@@ -4756,8 +4966,10 @@
       <c r="M96" s="11"/>
       <c r="N96" s="11"/>
       <c r="O96" s="11"/>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P96" s="11"/>
+      <c r="Q96" s="11"/>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="11">
         <v>2011</v>
       </c>
@@ -4793,8 +5005,10 @@
       <c r="M97" s="11"/>
       <c r="N97" s="11"/>
       <c r="O97" s="11"/>
-    </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P97" s="11"/>
+      <c r="Q97" s="11"/>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="11">
         <v>2011</v>
       </c>
@@ -4830,8 +5044,10 @@
       <c r="M98" s="11"/>
       <c r="N98" s="11"/>
       <c r="O98" s="11"/>
-    </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P98" s="11"/>
+      <c r="Q98" s="11"/>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="11">
         <v>2011</v>
       </c>
@@ -4867,8 +5083,10 @@
       <c r="M99" s="11"/>
       <c r="N99" s="11"/>
       <c r="O99" s="11"/>
-    </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P99" s="11"/>
+      <c r="Q99" s="11"/>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="11">
         <v>2011</v>
       </c>
@@ -4904,8 +5122,10 @@
       <c r="M100" s="11"/>
       <c r="N100" s="11"/>
       <c r="O100" s="11"/>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P100" s="11"/>
+      <c r="Q100" s="11"/>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="11">
         <v>2011</v>
       </c>
@@ -4941,8 +5161,10 @@
       <c r="M101" s="11"/>
       <c r="N101" s="11"/>
       <c r="O101" s="11"/>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P101" s="11"/>
+      <c r="Q101" s="11"/>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="11">
         <v>2011</v>
       </c>
@@ -4978,8 +5200,10 @@
       <c r="M102" s="11"/>
       <c r="N102" s="11"/>
       <c r="O102" s="11"/>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P102" s="11"/>
+      <c r="Q102" s="11"/>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="12">
         <v>2012</v>
       </c>
@@ -5015,8 +5239,10 @@
       <c r="M103" s="12"/>
       <c r="N103" s="12"/>
       <c r="O103" s="12"/>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P103" s="12"/>
+      <c r="Q103" s="12"/>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="12">
         <v>2012</v>
       </c>
@@ -5052,8 +5278,10 @@
       <c r="M104" s="12"/>
       <c r="N104" s="12"/>
       <c r="O104" s="12"/>
-    </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P104" s="12"/>
+      <c r="Q104" s="12"/>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="12">
         <v>2012</v>
       </c>
@@ -5091,8 +5319,10 @@
       <c r="M105" s="12"/>
       <c r="N105" s="12"/>
       <c r="O105" s="12"/>
-    </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P105" s="12"/>
+      <c r="Q105" s="12"/>
+    </row>
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="12">
         <v>2012</v>
       </c>
@@ -5128,8 +5358,10 @@
       <c r="M106" s="12"/>
       <c r="N106" s="12"/>
       <c r="O106" s="12"/>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P106" s="12"/>
+      <c r="Q106" s="12"/>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="12">
         <v>2012</v>
       </c>
@@ -5167,8 +5399,10 @@
       <c r="M107" s="12"/>
       <c r="N107" s="12"/>
       <c r="O107" s="12"/>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P107" s="12"/>
+      <c r="Q107" s="12"/>
+    </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="12">
         <v>2012</v>
       </c>
@@ -5206,8 +5440,10 @@
       <c r="M108" s="12"/>
       <c r="N108" s="12"/>
       <c r="O108" s="12"/>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P108" s="12"/>
+      <c r="Q108" s="12"/>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="12">
         <v>2012</v>
       </c>
@@ -5240,8 +5476,10 @@
       <c r="M109" s="12"/>
       <c r="N109" s="12"/>
       <c r="O109" s="12"/>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P109" s="12"/>
+      <c r="Q109" s="12"/>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="12">
         <v>2012</v>
       </c>
@@ -5274,8 +5512,10 @@
       <c r="M110" s="12"/>
       <c r="N110" s="12"/>
       <c r="O110" s="12"/>
-    </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P110" s="12"/>
+      <c r="Q110" s="12"/>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="12">
         <v>2012</v>
       </c>
@@ -5311,8 +5551,10 @@
       <c r="M111" s="12"/>
       <c r="N111" s="12"/>
       <c r="O111" s="12"/>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P111" s="12"/>
+      <c r="Q111" s="12"/>
+    </row>
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="12">
         <v>2012</v>
       </c>
@@ -5350,8 +5592,10 @@
       <c r="M112" s="12"/>
       <c r="N112" s="12"/>
       <c r="O112" s="12"/>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P112" s="12"/>
+      <c r="Q112" s="12"/>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="12">
         <v>2012</v>
       </c>
@@ -5387,8 +5631,10 @@
       <c r="M113" s="12"/>
       <c r="N113" s="12"/>
       <c r="O113" s="12"/>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P113" s="12"/>
+      <c r="Q113" s="12"/>
+    </row>
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="12">
         <v>2012</v>
       </c>
@@ -5426,8 +5672,10 @@
       <c r="M114" s="12"/>
       <c r="N114" s="12"/>
       <c r="O114" s="12"/>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P114" s="12"/>
+      <c r="Q114" s="12"/>
+    </row>
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" s="12">
         <v>2012</v>
       </c>
@@ -5465,8 +5713,10 @@
       <c r="M115" s="12"/>
       <c r="N115" s="12"/>
       <c r="O115" s="12"/>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P115" s="12"/>
+      <c r="Q115" s="12"/>
+    </row>
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" s="12">
         <v>2012</v>
       </c>
@@ -5502,8 +5752,10 @@
       <c r="M116" s="12"/>
       <c r="N116" s="12"/>
       <c r="O116" s="12"/>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P116" s="12"/>
+      <c r="Q116" s="12"/>
+    </row>
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="12">
         <v>2012</v>
       </c>
@@ -5539,8 +5791,10 @@
       <c r="M117" s="12"/>
       <c r="N117" s="12"/>
       <c r="O117" s="12"/>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P117" s="12"/>
+      <c r="Q117" s="12"/>
+    </row>
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" s="12">
         <v>2012</v>
       </c>
@@ -5578,8 +5832,10 @@
       <c r="M118" s="12"/>
       <c r="N118" s="12"/>
       <c r="O118" s="12"/>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P118" s="12"/>
+      <c r="Q118" s="12"/>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" s="12">
         <v>2012</v>
       </c>
@@ -5615,8 +5871,10 @@
       <c r="M119" s="12"/>
       <c r="N119" s="12"/>
       <c r="O119" s="12"/>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P119" s="12"/>
+      <c r="Q119" s="12"/>
+    </row>
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="12">
         <v>2012</v>
       </c>
@@ -5652,8 +5910,10 @@
       <c r="M120" s="12"/>
       <c r="N120" s="12"/>
       <c r="O120" s="12"/>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P120" s="12"/>
+      <c r="Q120" s="12"/>
+    </row>
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="12">
         <v>2012</v>
       </c>
@@ -5686,8 +5946,10 @@
       <c r="M121" s="12"/>
       <c r="N121" s="12"/>
       <c r="O121" s="12"/>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P121" s="12"/>
+      <c r="Q121" s="12"/>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" s="12">
         <v>2012</v>
       </c>
@@ -5723,8 +5985,10 @@
       <c r="M122" s="12"/>
       <c r="N122" s="12"/>
       <c r="O122" s="12"/>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P122" s="12"/>
+      <c r="Q122" s="12"/>
+    </row>
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" s="12">
         <v>2012</v>
       </c>
@@ -5760,8 +6024,10 @@
       <c r="M123" s="12"/>
       <c r="N123" s="12"/>
       <c r="O123" s="12"/>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P123" s="12"/>
+      <c r="Q123" s="12"/>
+    </row>
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" s="12">
         <v>2012</v>
       </c>
@@ -5797,8 +6063,10 @@
       <c r="M124" s="12"/>
       <c r="N124" s="12"/>
       <c r="O124" s="12"/>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P124" s="12"/>
+      <c r="Q124" s="12"/>
+    </row>
+    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" s="12">
         <v>2012</v>
       </c>
@@ -5834,8 +6102,10 @@
       <c r="M125" s="12"/>
       <c r="N125" s="12"/>
       <c r="O125" s="12"/>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P125" s="12"/>
+      <c r="Q125" s="12"/>
+    </row>
+    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>2013</v>
       </c>
@@ -5871,8 +6141,10 @@
       <c r="M126" s="1"/>
       <c r="N126" s="1"/>
       <c r="O126" s="1"/>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P126" s="1"/>
+      <c r="Q126" s="1"/>
+    </row>
+    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>2013</v>
       </c>
@@ -5906,8 +6178,10 @@
       <c r="M127" s="1"/>
       <c r="N127" s="1"/>
       <c r="O127" s="1"/>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P127" s="1"/>
+      <c r="Q127" s="1"/>
+    </row>
+    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>2013</v>
       </c>
@@ -5941,8 +6215,10 @@
       <c r="M128" s="1"/>
       <c r="N128" s="1"/>
       <c r="O128" s="1"/>
-    </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P128" s="1"/>
+      <c r="Q128" s="1"/>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>2013</v>
       </c>
@@ -5976,8 +6252,10 @@
       <c r="M129" s="1"/>
       <c r="N129" s="1"/>
       <c r="O129" s="1"/>
-    </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P129" s="1"/>
+      <c r="Q129" s="1"/>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>2013</v>
       </c>
@@ -6011,8 +6289,10 @@
       <c r="M130" s="1"/>
       <c r="N130" s="1"/>
       <c r="O130" s="1"/>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P130" s="1"/>
+      <c r="Q130" s="1"/>
+    </row>
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>2013</v>
       </c>
@@ -6046,8 +6326,10 @@
       <c r="M131" s="1"/>
       <c r="N131" s="1"/>
       <c r="O131" s="1"/>
-    </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P131" s="1"/>
+      <c r="Q131" s="1"/>
+    </row>
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>2013</v>
       </c>
@@ -6083,8 +6365,10 @@
       <c r="M132" s="1"/>
       <c r="N132" s="1"/>
       <c r="O132" s="1"/>
-    </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P132" s="1"/>
+      <c r="Q132" s="1"/>
+    </row>
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>2013</v>
       </c>
@@ -6120,8 +6404,10 @@
       <c r="M133" s="1"/>
       <c r="N133" s="1"/>
       <c r="O133" s="1"/>
-    </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P133" s="1"/>
+      <c r="Q133" s="1"/>
+    </row>
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="6">
         <v>2014</v>
       </c>
@@ -6159,8 +6445,10 @@
       <c r="M134" s="6"/>
       <c r="N134" s="6"/>
       <c r="O134" s="6"/>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P134" s="6"/>
+      <c r="Q134" s="6"/>
+    </row>
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" s="6">
         <v>2014</v>
       </c>
@@ -6200,8 +6488,10 @@
       <c r="M135" s="6"/>
       <c r="N135" s="6"/>
       <c r="O135" s="6"/>
-    </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P135" s="6"/>
+      <c r="Q135" s="6"/>
+    </row>
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" s="6">
         <v>2014</v>
       </c>
@@ -6241,8 +6531,10 @@
       <c r="M136" s="6"/>
       <c r="N136" s="6"/>
       <c r="O136" s="6"/>
-    </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P136" s="6"/>
+      <c r="Q136" s="6"/>
+    </row>
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" s="6">
         <v>2014</v>
       </c>
@@ -6280,8 +6572,10 @@
       <c r="M137" s="6"/>
       <c r="N137" s="6"/>
       <c r="O137" s="6"/>
-    </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P137" s="6"/>
+      <c r="Q137" s="6"/>
+    </row>
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" s="6">
         <v>2014</v>
       </c>
@@ -6319,8 +6613,10 @@
       <c r="M138" s="6"/>
       <c r="N138" s="6"/>
       <c r="O138" s="6"/>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P138" s="6"/>
+      <c r="Q138" s="6"/>
+    </row>
+    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="6">
         <v>2014</v>
       </c>
@@ -6356,8 +6652,10 @@
       <c r="M139" s="6"/>
       <c r="N139" s="6"/>
       <c r="O139" s="6"/>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P139" s="6"/>
+      <c r="Q139" s="6"/>
+    </row>
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" s="6">
         <v>2014</v>
       </c>
@@ -6397,8 +6695,10 @@
       <c r="M140" s="6"/>
       <c r="N140" s="6"/>
       <c r="O140" s="6"/>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P140" s="6"/>
+      <c r="Q140" s="6"/>
+    </row>
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" s="6">
         <v>2014</v>
       </c>
@@ -6434,8 +6734,10 @@
       <c r="M141" s="6"/>
       <c r="N141" s="6"/>
       <c r="O141" s="6"/>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P141" s="6"/>
+      <c r="Q141" s="6"/>
+    </row>
+    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" s="6">
         <v>2014</v>
       </c>
@@ -6473,8 +6775,10 @@
       <c r="M142" s="6"/>
       <c r="N142" s="6"/>
       <c r="O142" s="6"/>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P142" s="6"/>
+      <c r="Q142" s="6"/>
+    </row>
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" s="6">
         <v>2014</v>
       </c>
@@ -6512,8 +6816,10 @@
       <c r="M143" s="6"/>
       <c r="N143" s="6"/>
       <c r="O143" s="6"/>
-    </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P143" s="6"/>
+      <c r="Q143" s="6"/>
+    </row>
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" s="6">
         <v>2014</v>
       </c>
@@ -6551,8 +6857,10 @@
       <c r="M144" s="6"/>
       <c r="N144" s="6"/>
       <c r="O144" s="6"/>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P144" s="6"/>
+      <c r="Q144" s="6"/>
+    </row>
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" s="6">
         <v>2014</v>
       </c>
@@ -6592,8 +6900,10 @@
       <c r="M145" s="6"/>
       <c r="N145" s="6"/>
       <c r="O145" s="6"/>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P145" s="6"/>
+      <c r="Q145" s="6"/>
+    </row>
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" s="6">
         <v>2014</v>
       </c>
@@ -6633,8 +6943,10 @@
       <c r="M146" s="6"/>
       <c r="N146" s="6"/>
       <c r="O146" s="6"/>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P146" s="6"/>
+      <c r="Q146" s="6"/>
+    </row>
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" s="6">
         <v>2014</v>
       </c>
@@ -6672,8 +6984,10 @@
       <c r="M147" s="6"/>
       <c r="N147" s="6"/>
       <c r="O147" s="6"/>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P147" s="6"/>
+      <c r="Q147" s="6"/>
+    </row>
+    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148" s="14">
         <v>2015</v>
       </c>
@@ -6714,8 +7028,10 @@
       <c r="M148" s="19"/>
       <c r="N148" s="19"/>
       <c r="O148" s="19"/>
-    </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P148" s="19"/>
+      <c r="Q148" s="19"/>
+    </row>
+    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A149" s="14">
         <v>2015</v>
       </c>
@@ -6756,8 +7072,10 @@
       <c r="M149" s="19"/>
       <c r="N149" s="19"/>
       <c r="O149" s="19"/>
-    </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P149" s="19"/>
+      <c r="Q149" s="19"/>
+    </row>
+    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A150" s="14">
         <v>2015</v>
       </c>
@@ -6798,8 +7116,10 @@
       <c r="M150" s="19"/>
       <c r="N150" s="19"/>
       <c r="O150" s="19"/>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P150" s="19"/>
+      <c r="Q150" s="19"/>
+    </row>
+    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" s="14">
         <v>2015</v>
       </c>
@@ -6840,8 +7160,10 @@
       <c r="M151" s="19"/>
       <c r="N151" s="19"/>
       <c r="O151" s="19"/>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P151" s="19"/>
+      <c r="Q151" s="19"/>
+    </row>
+    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" s="14">
         <v>2015</v>
       </c>
@@ -6882,8 +7204,10 @@
       <c r="M152" s="19"/>
       <c r="N152" s="19"/>
       <c r="O152" s="19"/>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P152" s="19"/>
+      <c r="Q152" s="19"/>
+    </row>
+    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153" s="14">
         <v>2015</v>
       </c>
@@ -6924,8 +7248,10 @@
       <c r="M153" s="19"/>
       <c r="N153" s="19"/>
       <c r="O153" s="19"/>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P153" s="19"/>
+      <c r="Q153" s="19"/>
+    </row>
+    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154" s="14">
         <v>2015</v>
       </c>
@@ -6962,8 +7288,10 @@
       <c r="M154" s="19"/>
       <c r="N154" s="19"/>
       <c r="O154" s="19"/>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P154" s="19"/>
+      <c r="Q154" s="19"/>
+    </row>
+    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A155" s="14">
         <v>2015</v>
       </c>
@@ -7002,8 +7330,10 @@
       <c r="M155" s="19"/>
       <c r="N155" s="19"/>
       <c r="O155" s="19"/>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P155" s="19"/>
+      <c r="Q155" s="19"/>
+    </row>
+    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A156" s="14">
         <v>2015</v>
       </c>
@@ -7040,8 +7370,10 @@
       <c r="M156" s="19"/>
       <c r="N156" s="19"/>
       <c r="O156" s="19"/>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P156" s="19"/>
+      <c r="Q156" s="19"/>
+    </row>
+    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A157" s="14">
         <v>2015</v>
       </c>
@@ -7080,8 +7412,10 @@
       <c r="M157" s="19"/>
       <c r="N157" s="19"/>
       <c r="O157" s="19"/>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P157" s="19"/>
+      <c r="Q157" s="19"/>
+    </row>
+    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A158" s="14">
         <v>2015</v>
       </c>
@@ -7118,8 +7452,10 @@
       <c r="M158" s="19"/>
       <c r="N158" s="19"/>
       <c r="O158" s="19"/>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P158" s="19"/>
+      <c r="Q158" s="19"/>
+    </row>
+    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159" s="14">
         <v>2015</v>
       </c>
@@ -7156,8 +7492,10 @@
       <c r="M159" s="19"/>
       <c r="N159" s="19"/>
       <c r="O159" s="19"/>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P159" s="19"/>
+      <c r="Q159" s="19"/>
+    </row>
+    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" s="14">
         <v>2015</v>
       </c>
@@ -7196,8 +7534,10 @@
       <c r="M160" s="19"/>
       <c r="N160" s="19"/>
       <c r="O160" s="19"/>
-    </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P160" s="19"/>
+      <c r="Q160" s="19"/>
+    </row>
+    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" s="14">
         <v>2015</v>
       </c>
@@ -7234,8 +7574,10 @@
       <c r="M161" s="19"/>
       <c r="N161" s="19"/>
       <c r="O161" s="19"/>
-    </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P161" s="19"/>
+      <c r="Q161" s="19"/>
+    </row>
+    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" s="14">
         <v>2015</v>
       </c>
@@ -7274,8 +7616,10 @@
       <c r="M162" s="19"/>
       <c r="N162" s="19"/>
       <c r="O162" s="19"/>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P162" s="19"/>
+      <c r="Q162" s="19"/>
+    </row>
+    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" s="14">
         <v>2015</v>
       </c>
@@ -7314,8 +7658,10 @@
       <c r="M163" s="19"/>
       <c r="N163" s="19"/>
       <c r="O163" s="19"/>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P163" s="19"/>
+      <c r="Q163" s="19"/>
+    </row>
+    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" s="14">
         <v>2015</v>
       </c>
@@ -7356,8 +7702,10 @@
       <c r="M164" s="19"/>
       <c r="N164" s="19"/>
       <c r="O164" s="19"/>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P164" s="19"/>
+      <c r="Q164" s="19"/>
+    </row>
+    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" s="14">
         <v>2015</v>
       </c>
@@ -7396,8 +7744,10 @@
       <c r="M165" s="19"/>
       <c r="N165" s="19"/>
       <c r="O165" s="19"/>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P165" s="19"/>
+      <c r="Q165" s="19"/>
+    </row>
+    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" s="14">
         <v>2015</v>
       </c>
@@ -7434,8 +7784,10 @@
       <c r="M166" s="19"/>
       <c r="N166" s="19"/>
       <c r="O166" s="19"/>
-    </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P166" s="19"/>
+      <c r="Q166" s="19"/>
+    </row>
+    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A167" s="12">
         <v>2017</v>
       </c>
@@ -7473,8 +7825,10 @@
       <c r="M167" s="12"/>
       <c r="N167" s="12"/>
       <c r="O167" s="12"/>
-    </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P167" s="12"/>
+      <c r="Q167" s="12"/>
+    </row>
+    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168" s="12">
         <v>2017</v>
       </c>
@@ -7512,8 +7866,10 @@
       <c r="M168" s="12"/>
       <c r="N168" s="12"/>
       <c r="O168" s="12"/>
-    </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P168" s="12"/>
+      <c r="Q168" s="12"/>
+    </row>
+    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169" s="12">
         <v>2017</v>
       </c>
@@ -7549,8 +7905,10 @@
       <c r="M169" s="12"/>
       <c r="N169" s="12"/>
       <c r="O169" s="12"/>
-    </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P169" s="12"/>
+      <c r="Q169" s="12"/>
+    </row>
+    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170" s="12">
         <v>2017</v>
       </c>
@@ -7588,8 +7946,10 @@
       <c r="M170" s="12"/>
       <c r="N170" s="12"/>
       <c r="O170" s="12"/>
-    </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P170" s="12"/>
+      <c r="Q170" s="12"/>
+    </row>
+    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A171" s="12">
         <v>2017</v>
       </c>
@@ -7627,8 +7987,10 @@
       <c r="M171" s="12"/>
       <c r="N171" s="12"/>
       <c r="O171" s="12"/>
-    </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P171" s="12"/>
+      <c r="Q171" s="12"/>
+    </row>
+    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A172" s="12">
         <v>2017</v>
       </c>
@@ -7666,8 +8028,10 @@
       <c r="M172" s="12"/>
       <c r="N172" s="12"/>
       <c r="O172" s="12"/>
-    </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P172" s="12"/>
+      <c r="Q172" s="12"/>
+    </row>
+    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A173" s="12">
         <v>2017</v>
       </c>
@@ -7705,8 +8069,10 @@
       <c r="M173" s="12"/>
       <c r="N173" s="12"/>
       <c r="O173" s="12"/>
-    </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P173" s="12"/>
+      <c r="Q173" s="12"/>
+    </row>
+    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A174" s="12">
         <v>2017</v>
       </c>
@@ -7744,8 +8110,10 @@
       <c r="M174" s="12"/>
       <c r="N174" s="12"/>
       <c r="O174" s="12"/>
-    </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P174" s="12"/>
+      <c r="Q174" s="12"/>
+    </row>
+    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A175" s="12">
         <v>2017</v>
       </c>
@@ -7783,8 +8151,10 @@
       <c r="M175" s="12"/>
       <c r="N175" s="12"/>
       <c r="O175" s="12"/>
-    </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P175" s="12"/>
+      <c r="Q175" s="12"/>
+    </row>
+    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A176" s="12">
         <v>2017</v>
       </c>
@@ -7822,8 +8192,10 @@
       <c r="M176" s="12"/>
       <c r="N176" s="12"/>
       <c r="O176" s="12"/>
-    </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P176" s="12"/>
+      <c r="Q176" s="12"/>
+    </row>
+    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A177" s="12">
         <v>2017</v>
       </c>
@@ -7859,8 +8231,10 @@
       <c r="M177" s="12"/>
       <c r="N177" s="12"/>
       <c r="O177" s="12"/>
-    </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P177" s="12"/>
+      <c r="Q177" s="12"/>
+    </row>
+    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A178" s="6">
         <v>2019</v>
       </c>
@@ -7894,8 +8268,10 @@
       <c r="M178" s="6"/>
       <c r="N178" s="6"/>
       <c r="O178" s="6"/>
-    </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P178" s="6"/>
+      <c r="Q178" s="6"/>
+    </row>
+    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A179" s="6">
         <v>2019</v>
       </c>
@@ -7931,8 +8307,10 @@
       <c r="M179" s="6"/>
       <c r="N179" s="6"/>
       <c r="O179" s="6"/>
-    </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P179" s="6"/>
+      <c r="Q179" s="6"/>
+    </row>
+    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A180" s="6">
         <v>2019</v>
       </c>
@@ -7968,8 +8346,10 @@
       <c r="M180" s="6"/>
       <c r="N180" s="6"/>
       <c r="O180" s="6"/>
-    </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P180" s="6"/>
+      <c r="Q180" s="6"/>
+    </row>
+    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A181" s="6">
         <v>2019</v>
       </c>
@@ -8005,8 +8385,10 @@
       <c r="M181" s="6"/>
       <c r="N181" s="6"/>
       <c r="O181" s="6"/>
-    </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P181" s="6"/>
+      <c r="Q181" s="6"/>
+    </row>
+    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A182" s="6">
         <v>2019</v>
       </c>
@@ -8042,8 +8424,10 @@
       <c r="M182" s="6"/>
       <c r="N182" s="6"/>
       <c r="O182" s="6"/>
-    </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P182" s="6"/>
+      <c r="Q182" s="6"/>
+    </row>
+    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A183" s="6">
         <v>2019</v>
       </c>
@@ -8079,8 +8463,10 @@
       <c r="M183" s="6"/>
       <c r="N183" s="6"/>
       <c r="O183" s="6"/>
-    </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P183" s="6"/>
+      <c r="Q183" s="6"/>
+    </row>
+    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A184" s="6">
         <v>2019</v>
       </c>
@@ -8116,8 +8502,10 @@
       <c r="M184" s="6"/>
       <c r="N184" s="6"/>
       <c r="O184" s="6"/>
-    </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P184" s="6"/>
+      <c r="Q184" s="6"/>
+    </row>
+    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A185" s="6">
         <v>2019</v>
       </c>
@@ -8149,8 +8537,10 @@
       <c r="M185" s="6"/>
       <c r="N185" s="6"/>
       <c r="O185" s="6"/>
-    </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P185" s="6"/>
+      <c r="Q185" s="6"/>
+    </row>
+    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A186" s="6">
         <v>2019</v>
       </c>
@@ -8186,8 +8576,10 @@
       <c r="M186" s="6"/>
       <c r="N186" s="6"/>
       <c r="O186" s="6"/>
-    </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P186" s="6"/>
+      <c r="Q186" s="6"/>
+    </row>
+    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A187" s="6">
         <v>2019</v>
       </c>
@@ -8223,8 +8615,10 @@
       <c r="M187" s="6"/>
       <c r="N187" s="6"/>
       <c r="O187" s="6"/>
-    </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P187" s="6"/>
+      <c r="Q187" s="6"/>
+    </row>
+    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A188" s="6">
         <v>2019</v>
       </c>
@@ -8260,8 +8654,10 @@
       <c r="M188" s="6"/>
       <c r="N188" s="6"/>
       <c r="O188" s="6"/>
-    </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P188" s="6"/>
+      <c r="Q188" s="6"/>
+    </row>
+    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189" s="6">
         <v>2019</v>
       </c>
@@ -8297,8 +8693,10 @@
       <c r="M189" s="6"/>
       <c r="N189" s="6"/>
       <c r="O189" s="6"/>
-    </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P189" s="6"/>
+      <c r="Q189" s="6"/>
+    </row>
+    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190" s="6">
         <v>2019</v>
       </c>
@@ -8334,8 +8732,10 @@
       <c r="M190" s="6"/>
       <c r="N190" s="6"/>
       <c r="O190" s="6"/>
-    </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P190" s="6"/>
+      <c r="Q190" s="6"/>
+    </row>
+    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191" s="6">
         <v>2019</v>
       </c>
@@ -8371,8 +8771,10 @@
       <c r="M191" s="6"/>
       <c r="N191" s="6"/>
       <c r="O191" s="6"/>
-    </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P191" s="6"/>
+      <c r="Q191" s="6"/>
+    </row>
+    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192" s="6">
         <v>2019</v>
       </c>
@@ -8404,8 +8806,10 @@
       <c r="M192" s="6"/>
       <c r="N192" s="6"/>
       <c r="O192" s="6"/>
-    </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P192" s="6"/>
+      <c r="Q192" s="6"/>
+    </row>
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="6">
         <v>2019</v>
       </c>
@@ -8437,8 +8841,10 @@
       <c r="M193" s="6"/>
       <c r="N193" s="6"/>
       <c r="O193" s="6"/>
-    </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P193" s="6"/>
+      <c r="Q193" s="6"/>
+    </row>
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="6">
         <v>2019</v>
       </c>
@@ -8470,8 +8876,10 @@
       <c r="M194" s="6"/>
       <c r="N194" s="6"/>
       <c r="O194" s="6"/>
-    </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P194" s="6"/>
+      <c r="Q194" s="6"/>
+    </row>
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="6">
         <v>2019</v>
       </c>
@@ -8503,8 +8911,10 @@
       <c r="M195" s="6"/>
       <c r="N195" s="6"/>
       <c r="O195" s="6"/>
-    </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P195" s="6"/>
+      <c r="Q195" s="6"/>
+    </row>
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="6">
         <v>2019</v>
       </c>
@@ -8538,8 +8948,10 @@
       <c r="M196" s="6"/>
       <c r="N196" s="6"/>
       <c r="O196" s="6"/>
-    </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P196" s="6"/>
+      <c r="Q196" s="6"/>
+    </row>
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="22">
         <v>2016</v>
       </c>
@@ -8580,8 +8992,10 @@
       <c r="M197" s="22"/>
       <c r="N197" s="22"/>
       <c r="O197" s="22"/>
-    </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P197" s="22"/>
+      <c r="Q197" s="22"/>
+    </row>
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="22">
         <v>2016</v>
       </c>
@@ -8618,8 +9032,10 @@
       <c r="M198" s="22"/>
       <c r="N198" s="22"/>
       <c r="O198" s="22"/>
-    </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P198" s="22"/>
+      <c r="Q198" s="22"/>
+    </row>
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="22">
         <v>2016</v>
       </c>
@@ -8658,8 +9074,10 @@
       <c r="M199" s="22"/>
       <c r="N199" s="22"/>
       <c r="O199" s="22"/>
-    </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P199" s="22"/>
+      <c r="Q199" s="22"/>
+    </row>
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="22">
         <v>2016</v>
       </c>
@@ -8694,8 +9112,10 @@
       <c r="M200" s="22"/>
       <c r="N200" s="22"/>
       <c r="O200" s="22"/>
-    </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P200" s="22"/>
+      <c r="Q200" s="22"/>
+    </row>
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" s="22">
         <v>2016</v>
       </c>
@@ -8734,8 +9154,10 @@
       <c r="M201" s="22"/>
       <c r="N201" s="22"/>
       <c r="O201" s="22"/>
-    </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P201" s="22"/>
+      <c r="Q201" s="22"/>
+    </row>
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" s="22">
         <v>2016</v>
       </c>
@@ -8772,8 +9194,10 @@
       <c r="M202" s="22"/>
       <c r="N202" s="22"/>
       <c r="O202" s="22"/>
-    </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P202" s="22"/>
+      <c r="Q202" s="22"/>
+    </row>
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A203" s="22">
         <v>2016</v>
       </c>
@@ -8812,8 +9236,10 @@
       <c r="M203" s="22"/>
       <c r="N203" s="22"/>
       <c r="O203" s="22"/>
-    </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P203" s="22"/>
+      <c r="Q203" s="22"/>
+    </row>
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A204" s="22">
         <v>2016</v>
       </c>
@@ -8850,8 +9276,10 @@
       <c r="M204" s="22"/>
       <c r="N204" s="22"/>
       <c r="O204" s="22"/>
-    </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P204" s="22"/>
+      <c r="Q204" s="22"/>
+    </row>
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A205" s="22">
         <v>2016</v>
       </c>
@@ -8890,8 +9318,10 @@
       <c r="M205" s="22"/>
       <c r="N205" s="22"/>
       <c r="O205" s="22"/>
-    </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P205" s="22"/>
+      <c r="Q205" s="22"/>
+    </row>
+    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A206" s="22">
         <v>2016</v>
       </c>
@@ -8930,8 +9360,10 @@
       <c r="M206" s="22"/>
       <c r="N206" s="22"/>
       <c r="O206" s="22"/>
-    </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P206" s="22"/>
+      <c r="Q206" s="22"/>
+    </row>
+    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A207" s="22">
         <v>2016</v>
       </c>
@@ -8968,8 +9400,10 @@
       <c r="M207" s="22"/>
       <c r="N207" s="22"/>
       <c r="O207" s="22"/>
-    </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P207" s="22"/>
+      <c r="Q207" s="22"/>
+    </row>
+    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A208" s="22">
         <v>2016</v>
       </c>
@@ -9006,8 +9440,10 @@
       <c r="M208" s="22"/>
       <c r="N208" s="22"/>
       <c r="O208" s="22"/>
-    </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P208" s="22"/>
+      <c r="Q208" s="22"/>
+    </row>
+    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A209" s="22">
         <v>2016</v>
       </c>
@@ -9044,8 +9480,10 @@
       <c r="M209" s="22"/>
       <c r="N209" s="22"/>
       <c r="O209" s="22"/>
-    </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P209" s="22"/>
+      <c r="Q209" s="22"/>
+    </row>
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A210" s="22">
         <v>2016</v>
       </c>
@@ -9082,8 +9520,10 @@
       <c r="M210" s="22"/>
       <c r="N210" s="22"/>
       <c r="O210" s="22"/>
-    </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P210" s="22"/>
+      <c r="Q210" s="22"/>
+    </row>
+    <row r="211" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A211" s="22">
         <v>2016</v>
       </c>
@@ -9120,8 +9560,10 @@
       <c r="M211" s="22"/>
       <c r="N211" s="22"/>
       <c r="O211" s="22"/>
-    </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P211" s="22"/>
+      <c r="Q211" s="22"/>
+    </row>
+    <row r="212" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A212" s="22">
         <v>2016</v>
       </c>
@@ -9158,8 +9600,10 @@
       <c r="M212" s="22"/>
       <c r="N212" s="22"/>
       <c r="O212" s="22"/>
-    </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P212" s="22"/>
+      <c r="Q212" s="22"/>
+    </row>
+    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A213" s="22">
         <v>2016</v>
       </c>
@@ -9196,8 +9640,10 @@
       <c r="M213" s="22"/>
       <c r="N213" s="22"/>
       <c r="O213" s="22"/>
-    </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P213" s="22"/>
+      <c r="Q213" s="22"/>
+    </row>
+    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A214" s="22">
         <v>2016</v>
       </c>
@@ -9234,8 +9680,10 @@
       <c r="M214" s="22"/>
       <c r="N214" s="22"/>
       <c r="O214" s="22"/>
-    </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P214" s="22"/>
+      <c r="Q214" s="22"/>
+    </row>
+    <row r="215" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A215" s="22">
         <v>2016</v>
       </c>
@@ -9272,8 +9720,10 @@
       <c r="M215" s="22"/>
       <c r="N215" s="22"/>
       <c r="O215" s="22"/>
-    </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P215" s="22"/>
+      <c r="Q215" s="22"/>
+    </row>
+    <row r="216" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A216" s="12">
         <v>2023</v>
       </c>
@@ -9304,13 +9754,19 @@
       </c>
       <c r="K216" s="12"/>
       <c r="L216" s="12"/>
-      <c r="M216" s="39">
+      <c r="M216" s="35">
         <v>1</v>
       </c>
-      <c r="N216" s="12"/>
-      <c r="O216" s="12"/>
-    </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N216" s="35">
+        <v>1</v>
+      </c>
+      <c r="O216" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P216" s="12"/>
+      <c r="Q216" s="12"/>
+    </row>
+    <row r="217" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A217" s="12">
         <v>2023</v>
       </c>
@@ -9341,13 +9797,19 @@
       </c>
       <c r="K217" s="12"/>
       <c r="L217" s="12"/>
-      <c r="M217" s="39">
+      <c r="M217" s="35">
         <v>1</v>
       </c>
-      <c r="N217" s="12"/>
-      <c r="O217" s="12"/>
-    </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N217" s="35">
+        <v>1</v>
+      </c>
+      <c r="O217" s="35" t="s">
+        <v>367</v>
+      </c>
+      <c r="P217" s="12"/>
+      <c r="Q217" s="12"/>
+    </row>
+    <row r="218" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A218" s="12">
         <v>2023</v>
       </c>
@@ -9378,13 +9840,19 @@
       </c>
       <c r="K218" s="12"/>
       <c r="L218" s="12"/>
-      <c r="M218" s="39">
+      <c r="M218" s="35">
         <v>1</v>
       </c>
-      <c r="N218" s="12"/>
-      <c r="O218" s="12"/>
-    </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N218" s="35">
+        <v>1</v>
+      </c>
+      <c r="O218" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P218" s="12"/>
+      <c r="Q218" s="12"/>
+    </row>
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A219" s="12">
         <v>2023</v>
       </c>
@@ -9415,13 +9883,19 @@
       </c>
       <c r="K219" s="12"/>
       <c r="L219" s="12"/>
-      <c r="M219" s="39">
+      <c r="M219" s="35">
         <v>1</v>
       </c>
-      <c r="N219" s="12"/>
-      <c r="O219" s="12"/>
-    </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N219" s="35">
+        <v>1</v>
+      </c>
+      <c r="O219" s="35" t="s">
+        <v>368</v>
+      </c>
+      <c r="P219" s="12"/>
+      <c r="Q219" s="12"/>
+    </row>
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A220" s="12">
         <v>2023</v>
       </c>
@@ -9452,13 +9926,19 @@
       </c>
       <c r="K220" s="12"/>
       <c r="L220" s="12"/>
-      <c r="M220" s="39">
+      <c r="M220" s="35">
         <v>1</v>
       </c>
-      <c r="N220" s="12"/>
-      <c r="O220" s="12"/>
-    </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N220" s="35">
+        <v>1</v>
+      </c>
+      <c r="O220" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P220" s="12"/>
+      <c r="Q220" s="12"/>
+    </row>
+    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A221" s="12">
         <v>2023</v>
       </c>
@@ -9489,13 +9969,19 @@
       </c>
       <c r="K221" s="12"/>
       <c r="L221" s="12"/>
-      <c r="M221" s="39">
+      <c r="M221" s="35">
         <v>0</v>
       </c>
-      <c r="N221" s="12"/>
-      <c r="O221" s="12"/>
-    </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N221" s="35">
+        <v>0</v>
+      </c>
+      <c r="O221" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P221" s="12"/>
+      <c r="Q221" s="12"/>
+    </row>
+    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A222" s="12">
         <v>2023</v>
       </c>
@@ -9526,13 +10012,19 @@
       </c>
       <c r="K222" s="12"/>
       <c r="L222" s="12"/>
-      <c r="M222" s="39">
+      <c r="M222" s="35">
         <v>1</v>
       </c>
-      <c r="N222" s="12"/>
-      <c r="O222" s="12"/>
-    </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N222" s="35">
+        <v>1</v>
+      </c>
+      <c r="O222" s="35" t="s">
+        <v>367</v>
+      </c>
+      <c r="P222" s="12"/>
+      <c r="Q222" s="12"/>
+    </row>
+    <row r="223" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A223" s="12">
         <v>2023</v>
       </c>
@@ -9563,13 +10055,19 @@
       </c>
       <c r="K223" s="12"/>
       <c r="L223" s="12"/>
-      <c r="M223" s="39">
+      <c r="M223" s="35">
         <v>1</v>
       </c>
-      <c r="N223" s="12"/>
-      <c r="O223" s="12"/>
-    </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N223" s="35">
+        <v>1</v>
+      </c>
+      <c r="O223" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P223" s="12"/>
+      <c r="Q223" s="12"/>
+    </row>
+    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A224" s="12">
         <v>2023</v>
       </c>
@@ -9600,13 +10098,19 @@
       </c>
       <c r="K224" s="12"/>
       <c r="L224" s="12"/>
-      <c r="M224" s="39">
+      <c r="M224" s="35">
         <v>0</v>
       </c>
-      <c r="N224" s="12"/>
-      <c r="O224" s="12"/>
-    </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N224" s="35">
+        <v>0</v>
+      </c>
+      <c r="O224" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P224" s="12"/>
+      <c r="Q224" s="12"/>
+    </row>
+    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A225" s="12">
         <v>2023</v>
       </c>
@@ -9637,13 +10141,19 @@
       </c>
       <c r="K225" s="12"/>
       <c r="L225" s="12"/>
-      <c r="M225" s="39">
+      <c r="M225" s="35">
         <v>0</v>
       </c>
-      <c r="N225" s="12"/>
-      <c r="O225" s="12"/>
-    </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N225" s="35">
+        <v>0</v>
+      </c>
+      <c r="O225" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P225" s="12"/>
+      <c r="Q225" s="12"/>
+    </row>
+    <row r="226" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A226" s="12">
         <v>2023</v>
       </c>
@@ -9674,13 +10184,19 @@
       </c>
       <c r="K226" s="12"/>
       <c r="L226" s="12"/>
-      <c r="M226" s="39">
+      <c r="M226" s="35">
         <v>0</v>
       </c>
-      <c r="N226" s="12"/>
-      <c r="O226" s="12"/>
-    </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N226" s="35">
+        <v>0</v>
+      </c>
+      <c r="O226" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P226" s="12"/>
+      <c r="Q226" s="12"/>
+    </row>
+    <row r="227" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A227" s="12">
         <v>2023</v>
       </c>
@@ -9711,13 +10227,19 @@
       </c>
       <c r="K227" s="12"/>
       <c r="L227" s="12"/>
-      <c r="M227" s="39">
+      <c r="M227" s="35">
         <v>0</v>
       </c>
-      <c r="N227" s="12"/>
-      <c r="O227" s="12"/>
-    </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N227" s="35">
+        <v>0</v>
+      </c>
+      <c r="O227" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P227" s="12"/>
+      <c r="Q227" s="12"/>
+    </row>
+    <row r="228" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A228" s="12">
         <v>2023</v>
       </c>
@@ -9748,13 +10270,19 @@
       </c>
       <c r="K228" s="12"/>
       <c r="L228" s="12"/>
-      <c r="M228" s="39">
+      <c r="M228" s="35">
         <v>0</v>
       </c>
-      <c r="N228" s="12"/>
-      <c r="O228" s="12"/>
-    </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N228" s="35">
+        <v>0</v>
+      </c>
+      <c r="O228" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P228" s="12"/>
+      <c r="Q228" s="12"/>
+    </row>
+    <row r="229" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A229" s="12">
         <v>2023</v>
       </c>
@@ -9785,13 +10313,19 @@
       </c>
       <c r="K229" s="12"/>
       <c r="L229" s="12"/>
-      <c r="M229" s="39">
+      <c r="M229" s="35">
         <v>0</v>
       </c>
-      <c r="N229" s="12"/>
-      <c r="O229" s="12"/>
-    </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N229" s="35">
+        <v>0</v>
+      </c>
+      <c r="O229" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P229" s="12"/>
+      <c r="Q229" s="12"/>
+    </row>
+    <row r="230" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A230" s="12">
         <v>2023</v>
       </c>
@@ -9822,13 +10356,19 @@
       </c>
       <c r="K230" s="12"/>
       <c r="L230" s="12"/>
-      <c r="M230" s="39">
+      <c r="M230" s="35">
         <v>0</v>
       </c>
-      <c r="N230" s="12"/>
-      <c r="O230" s="12"/>
-    </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N230" s="35">
+        <v>0</v>
+      </c>
+      <c r="O230" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P230" s="12"/>
+      <c r="Q230" s="12"/>
+    </row>
+    <row r="231" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A231" s="12">
         <v>2023</v>
       </c>
@@ -9859,13 +10399,19 @@
       </c>
       <c r="K231" s="12"/>
       <c r="L231" s="12"/>
-      <c r="M231" s="39">
+      <c r="M231" s="35">
         <v>1</v>
       </c>
-      <c r="N231" s="12"/>
-      <c r="O231" s="12"/>
-    </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N231" s="35">
+        <v>1</v>
+      </c>
+      <c r="O231" s="35" t="s">
+        <v>368</v>
+      </c>
+      <c r="P231" s="12"/>
+      <c r="Q231" s="12"/>
+    </row>
+    <row r="232" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A232" s="12">
         <v>2023</v>
       </c>
@@ -9896,13 +10442,19 @@
       </c>
       <c r="K232" s="12"/>
       <c r="L232" s="12"/>
-      <c r="M232" s="39">
+      <c r="M232" s="35">
         <v>1</v>
       </c>
-      <c r="N232" s="12"/>
-      <c r="O232" s="12"/>
-    </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N232" s="35">
+        <v>0</v>
+      </c>
+      <c r="O232" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P232" s="12"/>
+      <c r="Q232" s="12"/>
+    </row>
+    <row r="233" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A233" s="12">
         <v>2023</v>
       </c>
@@ -9933,13 +10485,19 @@
       </c>
       <c r="K233" s="12"/>
       <c r="L233" s="12"/>
-      <c r="M233" s="39">
+      <c r="M233" s="35">
         <v>0</v>
       </c>
-      <c r="N233" s="12"/>
-      <c r="O233" s="12"/>
-    </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N233" s="35">
+        <v>0</v>
+      </c>
+      <c r="O233" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P233" s="12"/>
+      <c r="Q233" s="12"/>
+    </row>
+    <row r="234" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A234" s="12">
         <v>2023</v>
       </c>
@@ -9970,13 +10528,19 @@
       </c>
       <c r="K234" s="12"/>
       <c r="L234" s="12"/>
-      <c r="M234" s="39">
+      <c r="M234" s="35">
         <v>1</v>
       </c>
-      <c r="N234" s="12"/>
-      <c r="O234" s="12"/>
-    </row>
-    <row r="235" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N234" s="35">
+        <v>1</v>
+      </c>
+      <c r="O234" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P234" s="12"/>
+      <c r="Q234" s="12"/>
+    </row>
+    <row r="235" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A235" s="12">
         <v>2023</v>
       </c>
@@ -10007,13 +10571,19 @@
       </c>
       <c r="K235" s="12"/>
       <c r="L235" s="12"/>
-      <c r="M235" s="39">
+      <c r="M235" s="35">
         <v>1</v>
       </c>
-      <c r="N235" s="12"/>
-      <c r="O235" s="12"/>
-    </row>
-    <row r="236" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N235" s="35">
+        <v>1</v>
+      </c>
+      <c r="O235" s="35" t="s">
+        <v>366</v>
+      </c>
+      <c r="P235" s="12"/>
+      <c r="Q235" s="12"/>
+    </row>
+    <row r="236" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A236" s="12">
         <v>2023</v>
       </c>
@@ -10044,13 +10614,19 @@
       </c>
       <c r="K236" s="12"/>
       <c r="L236" s="12"/>
-      <c r="M236" s="39">
+      <c r="M236" s="35">
         <v>0</v>
       </c>
-      <c r="N236" s="12"/>
-      <c r="O236" s="12"/>
-    </row>
-    <row r="237" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N236" s="35">
+        <v>0</v>
+      </c>
+      <c r="O236" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P236" s="12"/>
+      <c r="Q236" s="12"/>
+    </row>
+    <row r="237" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A237" s="12">
         <v>2023</v>
       </c>
@@ -10081,13 +10657,19 @@
       </c>
       <c r="K237" s="12"/>
       <c r="L237" s="12"/>
-      <c r="M237" s="39">
+      <c r="M237" s="35">
         <v>0</v>
       </c>
-      <c r="N237" s="12"/>
-      <c r="O237" s="12"/>
-    </row>
-    <row r="238" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N237" s="35">
+        <v>0</v>
+      </c>
+      <c r="O237" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P237" s="12"/>
+      <c r="Q237" s="12"/>
+    </row>
+    <row r="238" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A238" s="12">
         <v>2023</v>
       </c>
@@ -10118,13 +10700,19 @@
       </c>
       <c r="K238" s="12"/>
       <c r="L238" s="12"/>
-      <c r="M238" s="39">
+      <c r="M238" s="35">
         <v>1</v>
       </c>
-      <c r="N238" s="12"/>
-      <c r="O238" s="12"/>
-    </row>
-    <row r="239" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N238" s="35">
+        <v>1</v>
+      </c>
+      <c r="O238" s="35" t="s">
+        <v>370</v>
+      </c>
+      <c r="P238" s="12"/>
+      <c r="Q238" s="12"/>
+    </row>
+    <row r="239" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A239" s="12">
         <v>2023</v>
       </c>
@@ -10155,13 +10743,19 @@
       </c>
       <c r="K239" s="12"/>
       <c r="L239" s="12"/>
-      <c r="M239" s="39">
+      <c r="M239" s="35">
         <v>0</v>
       </c>
-      <c r="N239" s="12"/>
-      <c r="O239" s="12"/>
-    </row>
-    <row r="240" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N239" s="35">
+        <v>0</v>
+      </c>
+      <c r="O239" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="P239" s="12"/>
+      <c r="Q239" s="12"/>
+    </row>
+    <row r="240" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A240" s="12">
         <v>2023</v>
       </c>
@@ -10192,13 +10786,19 @@
       </c>
       <c r="K240" s="12"/>
       <c r="L240" s="12"/>
-      <c r="M240" s="39">
+      <c r="M240" s="35">
         <v>1</v>
       </c>
-      <c r="N240" s="12"/>
-      <c r="O240" s="12"/>
-    </row>
-    <row r="241" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N240" s="35">
+        <v>1</v>
+      </c>
+      <c r="O240" s="35" t="s">
+        <v>370</v>
+      </c>
+      <c r="P240" s="12"/>
+      <c r="Q240" s="12"/>
+    </row>
+    <row r="241" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A241" s="12">
         <v>2023</v>
       </c>
@@ -10229,11 +10829,17 @@
       </c>
       <c r="K241" s="12"/>
       <c r="L241" s="12"/>
-      <c r="M241" s="39">
+      <c r="M241" s="35">
         <v>1</v>
       </c>
-      <c r="N241" s="12"/>
-      <c r="O241" s="12"/>
+      <c r="N241" s="35">
+        <v>1</v>
+      </c>
+      <c r="O241" s="35" t="s">
+        <v>371</v>
+      </c>
+      <c r="P241" s="12"/>
+      <c r="Q241" s="12"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">

</xml_diff>